<commit_message>
création des colonnes pour le fichier excel
</commit_message>
<xml_diff>
--- a/total_vente_trismestre.xlsx
+++ b/total_vente_trismestre.xlsx
@@ -345,13 +345,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Articles</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Octobre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Novembre</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Décembre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
commentaire du code précédent et création des noms des lignes de la première colonne "Article" à l'aide d'une boucle.
</commit_message>
<xml_diff>
--- a/total_vente_trismestre.xlsx
+++ b/total_vente_trismestre.xlsx
@@ -345,7 +345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -367,6 +367,34 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>Décembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pommes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dentifrice</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>manga berserk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Puce de téléphone</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
réecriture et décommentaire du code précédent car je vais l'utiliser
</commit_message>
<xml_diff>
--- a/total_vente_trismestre.xlsx
+++ b/total_vente_trismestre.xlsx
@@ -380,21 +380,21 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dentifrice</t>
+          <t>Poire</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>manga berserk</t>
+          <t>bannanemangue</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Puce de téléphone</t>
+          <t>Ananas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
rajout de la méthode de jonathan
</commit_message>
<xml_diff>
--- a/total_vente_trismestre.xlsx
+++ b/total_vente_trismestre.xlsx
@@ -345,7 +345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -376,26 +376,78 @@
           <t>Pommes</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>760</v>
+      </c>
+      <c r="C2" t="n">
+        <v>660</v>
+      </c>
+      <c r="D2" t="n">
+        <v>900</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Poire</t>
-        </is>
+          <t>Poires</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C3" t="n">
+        <v>625</v>
+      </c>
+      <c r="D3" t="n">
+        <v>594</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bannane</t>
-        </is>
+          <t>Bananes</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1440</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1170</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mangue</t>
-        </is>
+          <t>Mangues</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>900</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1125</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1254</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ananas</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>950</v>
+      </c>
+      <c r="C6" t="n">
+        <v>880</v>
+      </c>
+      <c r="D6" t="n">
+        <v>756</v>
       </c>
     </row>
   </sheetData>

</xml_diff>